<commit_message>
Apply 3 of the 5 pre-approved summary fixes (Phase 4c)
Ran scripts/apply_summary_fixes_2026-09-23.py --apply against the live
database. DPDPA-S6.9 and DPDPA-S27.1d's summaries now correctly say their
commencement is 6 months BEFORE the rest of their section (not "a year
after" — G.S.R. 843(E) clause (b) vs (c)). DPDPR-R12's summary now
correctly says Rule 12 exempts from both s.9(1) and s.9(3), not just the
tracking prohibition.

DPDPA-S44.2 and DPDPA-S44.1_3 were NOT touched: their current summaries
have already diverged from what the audit's fix was written against (an
earlier, unrelated rewrite changed them again since). Recorded as
change_origin='data_correction' (never highlighted, latest_change_id
untouched — verified: the Act docx still shows 0 highlights, the Rules
docx still shows exactly the 4 Phase 4a corrigendum highlights and
nothing new).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/DPDP_Rules_Tracker.xlsx
+++ b/data/DPDP_Rules_Tracker.xlsx
@@ -2011,7 +2011,7 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Every Consent Manager must be registered with the Board, subject to prescribed technical, operational, and financial conditions. (This sub-clause commences a year after the rest of Section 6, alongside Rule 4's registration process.)</t>
+          <t>Every Consent Manager must be registered with the Board, subject to prescribed technical, operational, financial and other conditions. (This sub-section commences one year after publication of G.S.R. 843(E) — six months BEFORE the rest of Section 6 — alongside Rule 4's registration process.)</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Exempts specified classes of Data Fiduciary (healthcare providers, educational institutions, crèches, child transport providers — Fourth Schedule Part A) and specified purposes (Part B, e.g. safety tracking, email accounts) from the Act's general prohibition on tracking/behavioural monitoring/targeted ads directed at children.</t>
+          <t>Exempts specified classes of Data Fiduciary (healthcare providers, educational institutions, crèches, child transport providers — Fourth Schedule Part A) and specified purposes (Part B, e.g. safety tracking, email accounts) from BOTH the verifiable parental consent requirement (s.9(1)) and the bar on tracking/behavioural monitoring/targeted ads directed at children (s.9(3)), subject to the Schedule's conditions.</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="J27" s="12" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="K27" s="12" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Gives the Board the power to inquire into, and penalise, a breach of Consent Manager registration conditions. (Commences a year after the rest of Section 27, alongside Section 6(9)'s Consent Manager registration requirement.)</t>
+          <t>Gives the Board the power to inquire into, and penalise, a breach of Consent Manager registration conditions. (Commences one year after publication of G.S.R. 843(E) — six months BEFORE the rest of Section 27 — alongside Section 6(9)'s Consent Manager registration requirement.)</t>
         </is>
       </c>
       <c r="F58" s="13" t="inlineStr">
@@ -7931,7 +7931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P140"/>
+  <dimension ref="A1:P143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17631,6 +17631,210 @@
       <c r="P140" s="12" t="inlineStr">
         <is>
           <t>Data-quality fix (not a regulatory change): restored text left out of DPDPR-SCH5 at seeding. See scripts/restore_rules_schedule_gaps_2026-09-23.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="12" t="inlineStr">
+        <is>
+          <t>CHG-0093</t>
+        </is>
+      </c>
+      <c r="B141" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-23T12:13:05.627930+00:00</t>
+        </is>
+      </c>
+      <c r="C141" s="12" t="inlineStr">
+        <is>
+          <t>DPDPA-S6.9</t>
+        </is>
+      </c>
+      <c r="D141" s="12" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="E141" s="12" t="inlineStr">
+        <is>
+          <t>data_correction</t>
+        </is>
+      </c>
+      <c r="F141" s="12" t="inlineStr">
+        <is>
+          <t>Every Consent Manager must be registered with the Board, subject to prescribed technical, operational, and financial conditions. (This sub-clause commences a year after the rest of Section 6, alongside Rule 4's registration process.)</t>
+        </is>
+      </c>
+      <c r="G141" s="12" t="inlineStr">
+        <is>
+          <t>Every Consent Manager must be registered with the Board, subject to prescribed technical, operational, financial and other conditions. (This sub-section commences one year after publication of G.S.R. 843(E) — six months BEFORE the rest of Section 6 — alongside Rule 4's registration process.)</t>
+        </is>
+      </c>
+      <c r="H141" s="12" t="inlineStr">
+        <is>
+          <t>Audit 2026-09-23</t>
+        </is>
+      </c>
+      <c r="I141" s="12" t="n"/>
+      <c r="J141" s="12" t="inlineStr">
+        <is>
+          <t>manual:audit-2026-09-23-summary-fix</t>
+        </is>
+      </c>
+      <c r="K141" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L141" s="12" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="M141" s="12" t="n"/>
+      <c r="N141" s="12" t="n"/>
+      <c r="O141" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P141" s="12" t="inlineStr">
+        <is>
+          <t>Summary-only data-quality fix (not a regulatory change; never highlighted). Basis: G.S.R. 843(E) clause (b) (one year) vs clause (c) (eighteen months: 'sub-sections (1) to (8) and (10) of section 6')</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="12" t="inlineStr">
+        <is>
+          <t>CHG-0094</t>
+        </is>
+      </c>
+      <c r="B142" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-23T12:13:05.627930+00:00</t>
+        </is>
+      </c>
+      <c r="C142" s="12" t="inlineStr">
+        <is>
+          <t>DPDPA-S27.1d</t>
+        </is>
+      </c>
+      <c r="D142" s="12" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="E142" s="12" t="inlineStr">
+        <is>
+          <t>data_correction</t>
+        </is>
+      </c>
+      <c r="F142" s="12" t="inlineStr">
+        <is>
+          <t>Gives the Board the power to inquire into, and penalise, a breach of Consent Manager registration conditions. (Commences a year after the rest of Section 27, alongside Section 6(9)'s Consent Manager registration requirement.)</t>
+        </is>
+      </c>
+      <c r="G142" s="12" t="inlineStr">
+        <is>
+          <t>Gives the Board the power to inquire into, and penalise, a breach of Consent Manager registration conditions. (Commences one year after publication of G.S.R. 843(E) — six months BEFORE the rest of Section 27 — alongside Section 6(9)'s Consent Manager registration requirement.)</t>
+        </is>
+      </c>
+      <c r="H142" s="12" t="inlineStr">
+        <is>
+          <t>Audit 2026-09-23</t>
+        </is>
+      </c>
+      <c r="I142" s="12" t="n"/>
+      <c r="J142" s="12" t="inlineStr">
+        <is>
+          <t>manual:audit-2026-09-23-summary-fix</t>
+        </is>
+      </c>
+      <c r="K142" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L142" s="12" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="M142" s="12" t="n"/>
+      <c r="N142" s="12" t="n"/>
+      <c r="O142" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P142" s="12" t="inlineStr">
+        <is>
+          <t>Summary-only data-quality fix (not a regulatory change; never highlighted). Basis: G.S.R. 843(E) clause (b) vs clause (c) ('section 27 except clause (d) of sub-section (1)')</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="12" t="inlineStr">
+        <is>
+          <t>CHG-0095</t>
+        </is>
+      </c>
+      <c r="B143" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-23T12:13:05.627930+00:00</t>
+        </is>
+      </c>
+      <c r="C143" s="12" t="inlineStr">
+        <is>
+          <t>DPDPR-R12</t>
+        </is>
+      </c>
+      <c r="D143" s="12" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="E143" s="12" t="inlineStr">
+        <is>
+          <t>data_correction</t>
+        </is>
+      </c>
+      <c r="F143" s="12" t="inlineStr">
+        <is>
+          <t>Exempts specified classes of Data Fiduciary (healthcare providers, educational institutions, crèches, child transport providers — Fourth Schedule Part A) and specified purposes (Part B, e.g. safety tracking, email accounts) from the Act's general prohibition on tracking/behavioural monitoring/targeted ads directed at children.</t>
+        </is>
+      </c>
+      <c r="G143" s="12" t="inlineStr">
+        <is>
+          <t>Exempts specified classes of Data Fiduciary (healthcare providers, educational institutions, crèches, child transport providers — Fourth Schedule Part A) and specified purposes (Part B, e.g. safety tracking, email accounts) from BOTH the verifiable parental consent requirement (s.9(1)) and the bar on tracking/behavioural monitoring/targeted ads directed at children (s.9(3)), subject to the Schedule's conditions.</t>
+        </is>
+      </c>
+      <c r="H143" s="12" t="inlineStr">
+        <is>
+          <t>Audit 2026-09-23</t>
+        </is>
+      </c>
+      <c r="I143" s="12" t="n"/>
+      <c r="J143" s="12" t="inlineStr">
+        <is>
+          <t>manual:audit-2026-09-23-summary-fix</t>
+        </is>
+      </c>
+      <c r="K143" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L143" s="12" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="M143" s="12" t="n"/>
+      <c r="N143" s="12" t="n"/>
+      <c r="O143" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P143" s="12" t="inlineStr">
+        <is>
+          <t>Summary-only data-quality fix (not a regulatory change; never highlighted). Basis: Rule 12(1),(2): 'The provisions of sub-sections (1) and (3) of section 9 of the Act shall not be applicable'</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate documents after the real pipeline run (Phase 8 final inspection)
Re-ran export_word.py and export_excel.py and inspected the output by
script, per Phase 8: Act docx has 0 highlighted runs; Rules docx
highlights exactly the 4 Phase 4a corrigendum words ("in the Official
Gazette" x2, "Departments", "order") and nothing else; Excel Change_Log
has exactly 3 yellow rows (CHG-0086/87/88, the corrigendum changes); the
README sheet's truthfulness spot-checked. The Excel tracker's Source_Log
now also reflects SRC-0007 (PIB's RSS URL), added by the real pipeline
run in the previous commit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/DPDP_Rules_Tracker.xlsx
+++ b/data/DPDP_Rules_Tracker.xlsx
@@ -17863,7 +17863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17927,27 +17927,27 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>SRC-0002</t>
+          <t>SRC-0003</t>
         </is>
       </c>
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>MeitY</t>
+          <t>eGazette</t>
         </is>
       </c>
       <c r="C2" s="12" t="inlineStr">
         <is>
-          <t>Digital Personal Data Protection Act, 2023 (Act No. 22 of 2023)</t>
+          <t>Gazette Notification G.S.R. 843(E), 13 Nov 2025 (Act commencement schedule)</t>
         </is>
       </c>
       <c r="D2" s="12" t="inlineStr">
         <is>
-          <t>https://www.meity.gov.in/static/uploads/2024/06/2bf1f0e9f04e6fb4f8fef35e82c42aa5.pdf</t>
+          <t>https://www.meity.gov.in/static/uploads/2025/11/c56ceae6c383460ca69577428d36828b.pdf</t>
         </is>
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>2023-08-11</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr">
@@ -17974,69 +17974,65 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>SRC-0003</t>
+          <t>SRC-0001</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>eGazette</t>
+          <t>MeitY</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>Gazette Notification G.S.R. 843(E), 13 Nov 2025 (Act commencement schedule)</t>
+          <t>DPDP Rules, 2025 — MeitY PDF (G.S.R. 846(E))</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>https://www.meity.gov.in/static/uploads/2025/11/c56ceae6c383460ca69577428d36828b.pdf</t>
-        </is>
-      </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>2025-11-13</t>
-        </is>
-      </c>
+          <t>https://www.meity.gov.in/static/uploads/2025/11/53450e6e5dc0bfa85ebd78686cadad39.pdf</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="n"/>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>manual-seed-not-hashed</t>
+          <t>76094c7228c8dbff357281552fa2b052fe363303eb8b2c33ee5361d38883070d</t>
         </is>
       </c>
       <c r="H3" s="12" t="inlineStr">
         <is>
-          <t>Processed</t>
+          <t>No Change Detected</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>CHG-A0001,CHG-A0002,CHG-A0003,CHG-A0004,CHG-A0005,CHG-A0006,CHG-A0007,CHG-A0008,CHG-A0009,CHG-A0010,CHG-A0011,CHG-A0012,CHG-A0013,CHG-A0014,CHG-A0015,CHG-A0016,CHG-A0017,CHG-A0018,CHG-A0019,CHG-A0020,CHG-A0021,CHG-A0022,CHG-A0023,CHG-A0024,CHG-A0025,CHG-A0026,CHG-A0027,CHG-A0028,CHG-A0029,CHG-A0030,CHG-A0031,CHG-A0032,CHG-A0033,CHG-A0034,CHG-A0035,CHG-A0036,CHG-A0037,CHG-A0038,CHG-A0039,CHG-A0040,CHG-A0041,CHG-A0042,CHG-A0043,CHG-A0044,CHG-A0045,CHG-A0046,CHG-A0047,CHG-A0048</t>
+          <t>CHG-0002,CHG-0003,CHG-0004,CHG-0005,CHG-0006,CHG-0007,CHG-0008,CHG-0009,CHG-0010,CHG-0011,CHG-0012,CHG-0013,CHG-0014,CHG-0015,CHG-0016,CHG-0017,CHG-0018,CHG-0019,CHG-0020,CHG-0021,CHG-0022,CHG-0023,CHG-0024,CHG-0025,CHG-0026,CHG-0027,CHG-0028,CHG-0029,CHG-0030,CHG-0031,CHG-0032</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>SRC-0001</t>
+          <t>SRC-0004</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>MeitY</t>
+          <t>PIB</t>
         </is>
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>DPDP Rules, 2025 — MeitY PDF (G.S.R. 846(E))</t>
+          <t>PIB — All Press Releases (English)</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>https://www.meity.gov.in/static/uploads/2025/11/53450e6e5dc0bfa85ebd78686cadad39.pdf</t>
+          <t>https://www.pib.gov.in/allRel.aspx</t>
         </is>
       </c>
       <c r="E4" s="12" t="n"/>
@@ -18047,7 +18043,7 @@
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>76094c7228c8dbff357281552fa2b052fe363303eb8b2c33ee5361d38883070d</t>
+          <t>d38842055f43a4f6ee39929156a2c93772a0b128ba3ab14f887a64fcf1c77e89</t>
         </is>
       </c>
       <c r="H4" s="12" t="inlineStr">
@@ -18055,31 +18051,27 @@
           <t>No Change Detected</t>
         </is>
       </c>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>CHG-0002,CHG-0003,CHG-0004,CHG-0005,CHG-0006,CHG-0007,CHG-0008,CHG-0009,CHG-0010,CHG-0011,CHG-0012,CHG-0013,CHG-0014,CHG-0015,CHG-0016,CHG-0017,CHG-0018,CHG-0019,CHG-0020,CHG-0021,CHG-0022,CHG-0023,CHG-0024,CHG-0025,CHG-0026,CHG-0027,CHG-0028,CHG-0029,CHG-0030,CHG-0031,CHG-0032</t>
-        </is>
-      </c>
+      <c r="I4" s="12" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>SRC-0004</t>
+          <t>SRC-0005</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>PIB</t>
+          <t>eGazette</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>PIB — All Press Releases (English)</t>
+          <t>eGazette — Home (best-effort; no stable search endpoint confirmed)</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/allRel.aspx</t>
+          <t>https://egazette.gov.in/</t>
         </is>
       </c>
       <c r="E5" s="12" t="n"/>
@@ -18090,7 +18082,7 @@
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>d38842055f43a4f6ee39929156a2c93772a0b128ba3ab14f887a64fcf1c77e89</t>
+          <t>5804450f38f800c83d0849fd9ad445e103b5d70cd17603a0519ecf3b14ddc5d3</t>
         </is>
       </c>
       <c r="H5" s="12" t="inlineStr">
@@ -18103,22 +18095,22 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>SRC-0005</t>
+          <t>SRC-0002</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>eGazette</t>
+          <t>MeitY</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>eGazette — Home (best-effort; no stable search endpoint confirmed)</t>
+          <t>DPDP Act, 2023 — MeitY PDF</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>https://egazette.gov.in/</t>
+          <t>https://www.meity.gov.in/static/uploads/2024/06/2bf1f0e9f04e6fb4f8fef35e82c42aa5.pdf</t>
         </is>
       </c>
       <c r="E6" s="12" t="n"/>
@@ -18129,7 +18121,7 @@
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>ca96805449aa0e1eb65ff8f302650b129a742ad9902372ad6409b3dd18248582</t>
+          <t>f15bda1ff8065c68f8e1cc57c50616264afeb49d72cfc48d1e92a2a3c473c1d2</t>
         </is>
       </c>
       <c r="H6" s="12" t="inlineStr">
@@ -18137,7 +18129,11 @@
           <t>No Change Detected</t>
         </is>
       </c>
-      <c r="I6" s="12" t="n"/>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>CHG-A0001,CHG-A0002,CHG-A0003,CHG-A0004,CHG-A0005,CHG-A0006,CHG-A0007,CHG-A0008,CHG-A0009,CHG-A0010,CHG-A0011,CHG-A0012,CHG-A0013,CHG-A0014,CHG-A0015,CHG-A0016,CHG-A0017,CHG-A0018,CHG-A0019,CHG-A0020,CHG-A0021,CHG-A0022,CHG-A0023,CHG-A0024,CHG-A0025,CHG-A0026,CHG-A0027,CHG-A0028,CHG-A0029,CHG-A0030,CHG-A0031,CHG-A0032,CHG-A0033,CHG-A0034,CHG-A0035,CHG-A0036,CHG-A0037,CHG-A0038,CHG-A0039,CHG-A0040,CHG-A0041,CHG-A0042,CHG-A0043,CHG-A0044,CHG-A0045,CHG-A0046,CHG-A0047,CHG-A0048</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -18185,6 +18181,45 @@
           <t>CHG-0086,CHG-0087,CHG-0088</t>
         </is>
       </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>SRC-0007</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>PIB</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>PIB — All Press Releases RSS (English, national)</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/RssMain.aspx?ModId=6&amp;Mid=0&amp;reg=3&amp;lang=1</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>303646cc4c4bce1f12f990b273eedffaa3f1ba4df657ca84d5418879e39c79ef</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>No Change Detected</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>